<commit_message>
feat: re-run Site_4 and Site_1_9 with 1*9 sample location formatting
</commit_message>
<xml_diff>
--- a/Site_4/raw_data/Sieve_test_sample_4-9-10.xlsx
+++ b/Site_4/raw_data/Sieve_test_sample_4-9-10.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MELINDA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\003_PRESENTATIONS\28_THI_NGHIEM_FAFALAB\2026_Sieve_Analysis_Test\Site_4\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A20F6489-17FA-4A65-B1C1-D63839B85D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A2E7620-32FB-48A3-A82B-AEC29ECD7B14}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28845" yWindow="2325" windowWidth="15045" windowHeight="13710" xr2:uid="{5BF2A230-63A3-40BF-983D-FF5C3C9A446B}"/>
   </bookViews>
@@ -19,15 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -100,10 +91,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,25 +409,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{547094E5-B87E-4AC5-80D0-53DDDC8B8279}">
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -447,114 +438,200 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>10</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>310.18</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>345.42</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D4" s="1">
+        <f>C4-B4</f>
+        <v>35.240000000000009</v>
+      </c>
+      <c r="E4">
+        <f>ROUND((D4/$D$14)*100,2)</f>
+        <v>7.06</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>20</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>293.33999999999997</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>402.44</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D5" s="1">
+        <f t="shared" ref="D5:D13" si="0">C5-B5</f>
+        <v>109.10000000000002</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E13" si="1">ROUND((D5/$D$14)*100,2)</f>
+        <v>21.86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>30</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>315.48</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>369.2</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D6" s="1">
+        <f t="shared" si="0"/>
+        <v>53.71999999999997</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>10.76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>40</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>281.54000000000002</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <v>318.52</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D7" s="1">
+        <f t="shared" si="0"/>
+        <v>36.979999999999961</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>50</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>342.06</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <v>375.62</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D8" s="1">
+        <f t="shared" si="0"/>
+        <v>33.56</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>6.72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>60</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>331.1</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>343.62</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D9" s="1">
+        <f t="shared" si="0"/>
+        <v>12.519999999999982</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>2.5099999999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>80</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>328.32</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>355.4</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D10" s="1">
+        <f t="shared" si="0"/>
+        <v>27.079999999999984</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>100</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>314.66000000000003</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>330.2</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D11" s="1">
+        <f t="shared" si="0"/>
+        <v>15.539999999999964</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>200</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>305.39999999999998</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>350.34</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D12" s="1">
+        <f t="shared" si="0"/>
+        <v>44.94</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>9.01</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>347.28</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>477.64</v>
+      </c>
+      <c r="D13" s="1">
+        <f t="shared" si="0"/>
+        <v>130.36000000000001</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>26.12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D14" s="1">
+        <f>SUM(D4:D13)</f>
+        <v>499.03999999999991</v>
       </c>
     </row>
   </sheetData>

</xml_diff>